<commit_message>
syncing after finishing all baselines eval except sfa
</commit_message>
<xml_diff>
--- a/Claude outputs/DecVAE_revision_tracker.xlsx
+++ b/Claude outputs/DecVAE_revision_tracker.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="10400" tabRatio="500" activeTab="1"/>
+    <workbookView windowWidth="11950" windowHeight="10400" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -258,6 +258,9 @@
     <t>FD fixed frequency boundaries and generalisability</t>
   </si>
   <si>
+    <t>Text / Experiment</t>
+  </si>
+  <si>
     <t>MR-E</t>
   </si>
   <si>
@@ -292,9 +295,6 @@
   </si>
   <si>
     <t>Decomposition is an inductive bias, not a guarantee</t>
-  </si>
-  <si>
-    <t>Text / Experiment</t>
   </si>
   <si>
     <t>Aligns with our own view; state when it helps. We can argue that even when semantic factors are split across components, their combination achieves disentanglement. This could be set up as an experiment to show how emotion is distributed in VAEs vs DecVAEs (partially shown in the interpretability analysis with 3D contours)</t>
@@ -1333,7 +1333,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="47">
+  <fills count="48">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1403,6 +1403,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.25"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1746,7 +1752,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="16" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1770,16 +1776,16 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1788,89 +1794,89 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1901,62 +1907,72 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1968,7 +1984,7 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2506,398 +2522,398 @@
   </cols>
   <sheetData>
     <row r="1" ht="19" spans="1:2">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="39" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="40" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="41" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="38" t="s">
+      <c r="A7" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="42" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="39" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="39">
+      <c r="A8" s="43" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="43">
         <f>COUNTIF(Comments!G:G,"Not started")</f>
         <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="40" t="s">
+      <c r="A9" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="39">
+      <c r="B9" s="43">
         <f>COUNTIF(Comments!G:G,"Planned")</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="41" t="s">
+      <c r="A10" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="39">
+      <c r="B10" s="43">
         <f>COUNTIF(Comments!G:G,"In progress")</f>
         <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="42" t="s">
+      <c r="A11" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="39">
+      <c r="B11" s="43">
         <f>COUNTIF(Comments!G:G,"Blocked")</f>
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="39">
+      <c r="B12" s="43">
         <f>COUNTIF(Comments!G:G,"Done")</f>
         <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="44" t="s">
+      <c r="A13" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="39">
+      <c r="B13" s="43">
         <f>COUNTIF(Comments!G:G,"Dropped")</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="45" t="s">
+      <c r="A14" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="39">
+      <c r="B14" s="43">
         <f>COUNTIF(Comments!G:G,"Optional")</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" s="46" t="s">
+      <c r="A15" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="46">
+      <c r="B15" s="50">
         <f>COUNTA(Comments!A:A)-2</f>
         <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="37" t="s">
+      <c r="A18" s="41" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="38" t="s">
+      <c r="A19" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="38" t="s">
+      <c r="B19" s="42" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="39" t="s">
-        <v>6</v>
-      </c>
-      <c r="B20" s="39">
+      <c r="A20" s="43" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" s="43">
         <f>COUNTIF(Experiments!G:G,"Not started")</f>
         <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21" s="40" t="s">
+      <c r="A21" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="39">
+      <c r="B21" s="43">
         <f>COUNTIF(Experiments!G:G,"Planned")</f>
         <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="41" t="s">
+      <c r="A22" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="39">
+      <c r="B22" s="43">
         <f>COUNTIF(Experiments!G:G,"In progress")</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23" s="42" t="s">
+      <c r="A23" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="39">
+      <c r="B23" s="43">
         <f>COUNTIF(Experiments!G:G,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="43" t="s">
+      <c r="A24" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="B24" s="39">
+      <c r="B24" s="43">
         <f>COUNTIF(Experiments!G:G,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="44" t="s">
+      <c r="A25" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="B25" s="39">
+      <c r="B25" s="43">
         <f>COUNTIF(Experiments!G:G,"Dropped")</f>
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26" s="45" t="s">
+      <c r="A26" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="B26" s="39">
+      <c r="B26" s="43">
         <f>COUNTIF(Experiments!G:G,"Optional")</f>
         <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="46" t="s">
+      <c r="A27" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="B27" s="46">
+      <c r="B27" s="50">
         <f>COUNTA(Experiments!A:A)-2</f>
         <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="37" t="s">
+      <c r="A30" s="41" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="38" t="s">
+      <c r="A31" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="B31" s="38" t="s">
+      <c r="B31" s="42" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:2">
-      <c r="A32" s="39" t="s">
-        <v>6</v>
-      </c>
-      <c r="B32" s="39">
+      <c r="A32" s="43" t="s">
+        <v>6</v>
+      </c>
+      <c r="B32" s="43">
         <f>COUNTIF(Writing!E:E,"Not started")</f>
         <v>22</v>
       </c>
     </row>
     <row r="33" spans="1:2">
-      <c r="A33" s="40" t="s">
+      <c r="A33" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="B33" s="39">
+      <c r="B33" s="43">
         <f>COUNTIF(Writing!E:E,"Planned")</f>
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:2">
-      <c r="A34" s="41" t="s">
+      <c r="A34" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="B34" s="39">
+      <c r="B34" s="43">
         <f>COUNTIF(Writing!E:E,"In progress")</f>
         <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:2">
-      <c r="A35" s="42" t="s">
+      <c r="A35" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="B35" s="39">
+      <c r="B35" s="43">
         <f>COUNTIF(Writing!E:E,"Blocked")</f>
         <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:2">
-      <c r="A36" s="43" t="s">
+      <c r="A36" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="B36" s="39">
+      <c r="B36" s="43">
         <f>COUNTIF(Writing!E:E,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:2">
-      <c r="A37" s="44" t="s">
+      <c r="A37" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="B37" s="39">
+      <c r="B37" s="43">
         <f>COUNTIF(Writing!E:E,"Dropped")</f>
         <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:2">
-      <c r="A38" s="45" t="s">
+      <c r="A38" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="B38" s="39">
+      <c r="B38" s="43">
         <f>COUNTIF(Writing!E:E,"Optional")</f>
         <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:2">
-      <c r="A39" s="46" t="s">
+      <c r="A39" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="B39" s="46">
+      <c r="B39" s="50">
         <f>COUNTA(Writing!A:A)-2</f>
         <v>26</v>
       </c>
     </row>
     <row r="42" spans="1:2">
-      <c r="A42" s="37" t="s">
+      <c r="A42" s="41" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="43" spans="1:2">
-      <c r="A43" s="38" t="s">
+      <c r="A43" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="38" t="s">
+      <c r="B43" s="42" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="44" spans="1:2">
-      <c r="A44" s="39" t="s">
-        <v>6</v>
-      </c>
-      <c r="B44" s="39">
+      <c r="A44" s="43" t="s">
+        <v>6</v>
+      </c>
+      <c r="B44" s="43">
         <f>COUNTIF(Decisions!E:E,"Not started")</f>
         <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:2">
-      <c r="A45" s="40" t="s">
+      <c r="A45" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="B45" s="39">
+      <c r="B45" s="43">
         <f>COUNTIF(Decisions!E:E,"Planned")</f>
         <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:2">
-      <c r="A46" s="41" t="s">
+      <c r="A46" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="B46" s="39">
+      <c r="B46" s="43">
         <f>COUNTIF(Decisions!E:E,"In progress")</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:2">
-      <c r="A47" s="42" t="s">
+      <c r="A47" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="B47" s="39">
+      <c r="B47" s="43">
         <f>COUNTIF(Decisions!E:E,"Blocked")</f>
         <v>7</v>
       </c>
     </row>
     <row r="48" spans="1:2">
-      <c r="A48" s="43" t="s">
+      <c r="A48" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="B48" s="39">
+      <c r="B48" s="43">
         <f>COUNTIF(Decisions!E:E,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:6">
-      <c r="A49" s="44" t="s">
+      <c r="A49" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="B49" s="39">
+      <c r="B49" s="43">
         <f>COUNTIF(Decisions!E:E,"Dropped")</f>
         <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:6">
-      <c r="A50" s="45" t="s">
+      <c r="A50" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="B50" s="39">
+      <c r="B50" s="43">
         <f>COUNTIF(Decisions!E:E,"Optional")</f>
         <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:6">
-      <c r="A51" s="46" t="s">
+      <c r="A51" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="B51" s="46">
+      <c r="B51" s="50">
         <f>COUNTA(Decisions!A:A)-2</f>
         <v>7</v>
       </c>
     </row>
     <row r="54" spans="1:6">
-      <c r="A54" s="37" t="s">
+      <c r="A54" s="41" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" spans="1:6">
-      <c r="A55" s="47" t="s">
+      <c r="A55" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="B55" s="47"/>
-      <c r="C55" s="47"/>
-      <c r="D55" s="47"/>
-      <c r="E55" s="47"/>
-      <c r="F55" s="47"/>
+      <c r="B55" s="51"/>
+      <c r="C55" s="51"/>
+      <c r="D55" s="51"/>
+      <c r="E55" s="51"/>
+      <c r="F55" s="51"/>
     </row>
     <row r="56" spans="1:6">
-      <c r="A56" s="47"/>
-      <c r="B56" s="47"/>
-      <c r="C56" s="47"/>
-      <c r="D56" s="47"/>
-      <c r="E56" s="47"/>
-      <c r="F56" s="47"/>
+      <c r="A56" s="51"/>
+      <c r="B56" s="51"/>
+      <c r="C56" s="51"/>
+      <c r="D56" s="51"/>
+      <c r="E56" s="51"/>
+      <c r="F56" s="51"/>
     </row>
     <row r="57" spans="1:6">
-      <c r="A57" s="47"/>
-      <c r="B57" s="47"/>
-      <c r="C57" s="47"/>
-      <c r="D57" s="47"/>
-      <c r="E57" s="47"/>
-      <c r="F57" s="47"/>
+      <c r="A57" s="51"/>
+      <c r="B57" s="51"/>
+      <c r="C57" s="51"/>
+      <c r="D57" s="51"/>
+      <c r="E57" s="51"/>
+      <c r="F57" s="51"/>
     </row>
     <row r="58" spans="1:6">
-      <c r="A58" s="47"/>
-      <c r="B58" s="47"/>
-      <c r="C58" s="47"/>
-      <c r="D58" s="47"/>
-      <c r="E58" s="47"/>
-      <c r="F58" s="47"/>
+      <c r="A58" s="51"/>
+      <c r="B58" s="51"/>
+      <c r="C58" s="51"/>
+      <c r="D58" s="51"/>
+      <c r="E58" s="51"/>
+      <c r="F58" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2982,7 +2998,7 @@
       <c r="G4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I4" s="4" t="s">
@@ -3011,7 +3027,7 @@
       <c r="G5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="H5" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I5" s="4" t="s">
@@ -3127,7 +3143,7 @@
       <c r="G9" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I9" s="4" t="s">
@@ -3135,31 +3151,31 @@
       </c>
     </row>
     <row r="10" s="11" customFormat="1" spans="1:9">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="G10" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="H10" s="18" t="s">
+      <c r="G10" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="I10" s="19" t="s">
+      <c r="I10" s="21" t="s">
         <v>62</v>
       </c>
     </row>
@@ -3205,7 +3221,7 @@
       <c r="D12" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="E12" s="20" t="s">
+      <c r="E12" s="22" t="s">
         <v>56</v>
       </c>
       <c r="F12" s="5" t="s">
@@ -3214,45 +3230,45 @@
       <c r="G12" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H12" s="16" t="s">
+      <c r="H12" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I12" s="4" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
-      <c r="A13" s="3" t="s">
+    <row r="13" s="12" customFormat="1" ht="25" spans="1:9">
+      <c r="A13" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="E13" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="F13" s="5" t="s">
+      <c r="E13" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H13" s="16" t="s">
+      <c r="F13" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H13" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="I13" s="4" t="s">
-        <v>74</v>
+      <c r="I13" s="12" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>68</v>
@@ -3261,7 +3277,7 @@
         <v>37</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>39</v>
@@ -3269,19 +3285,19 @@
       <c r="F14" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="G14" s="21" t="s">
+      <c r="G14" s="23" t="s">
         <v>10</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>65</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>68</v>
@@ -3290,7 +3306,7 @@
         <v>37</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>39</v>
@@ -3305,93 +3321,93 @@
         <v>65</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="16" s="12" customFormat="1" ht="62.5" spans="1:9">
-      <c r="A16" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="B16" s="23" t="s">
+    </row>
+    <row r="16" s="13" customFormat="1" ht="62.5" spans="1:9">
+      <c r="A16" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="B16" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="D16" s="24" t="s">
+      <c r="C16" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="E16" s="23" t="s">
+      <c r="D16" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="F16" s="23" t="s">
+      <c r="E16" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="G16" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="H16" s="23" t="s">
+      <c r="F16" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="G16" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="H16" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="I16" s="24" t="s">
+      <c r="I16" s="12" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="17" s="12" customFormat="1" spans="1:9">
-      <c r="A17" s="22" t="s">
+    <row r="17" s="13" customFormat="1" spans="1:9">
+      <c r="A17" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="B17" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="C17" s="23" t="s">
+      <c r="B17" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D17" s="24" t="s">
+      <c r="D17" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="E17" s="23" t="s">
+      <c r="E17" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="F17" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="G17" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="H17" s="23" t="s">
+      <c r="F17" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="G17" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="H17" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="I17" s="24" t="s">
+      <c r="I17" s="12" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="18" s="12" customFormat="1" spans="1:9">
-      <c r="A18" s="22" t="s">
+    <row r="18" s="13" customFormat="1" spans="1:9">
+      <c r="A18" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="B18" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="C18" s="23" t="s">
+      <c r="B18" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D18" s="24" t="s">
+      <c r="D18" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="E18" s="23" t="s">
+      <c r="E18" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="F18" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="G18" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="H18" s="23" t="s">
+      <c r="F18" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="G18" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="H18" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="I18" s="24" t="s">
+      <c r="I18" s="12" t="s">
         <v>92</v>
       </c>
     </row>
@@ -3400,7 +3416,7 @@
         <v>93</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>37</v>
@@ -3429,7 +3445,7 @@
         <v>96</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>54</v>
@@ -3446,7 +3462,7 @@
       <c r="G20" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H20" s="16" t="s">
+      <c r="H20" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I20" s="4" t="s">
@@ -3458,7 +3474,7 @@
         <v>99</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>37</v>
@@ -3472,7 +3488,7 @@
       <c r="F21" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="21" t="s">
+      <c r="G21" s="23" t="s">
         <v>10</v>
       </c>
       <c r="H21" s="5" t="s">
@@ -3504,7 +3520,7 @@
       <c r="G22" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H22" s="16" t="s">
+      <c r="H22" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I22" s="4" t="s">
@@ -3524,7 +3540,7 @@
       <c r="D23" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="E23" s="20" t="s">
+      <c r="E23" s="22" t="s">
         <v>56</v>
       </c>
       <c r="F23" s="5" t="s">
@@ -3533,7 +3549,7 @@
       <c r="G23" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H23" s="16" t="s">
+      <c r="H23" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I23" s="4" t="s">
@@ -3591,7 +3607,7 @@
       <c r="G25" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H25" s="16" t="s">
+      <c r="H25" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I25" s="4" t="s">
@@ -3627,177 +3643,177 @@
         <v>120</v>
       </c>
     </row>
-    <row r="27" s="12" customFormat="1" spans="1:9">
-      <c r="A27" s="22" t="s">
+    <row r="27" s="13" customFormat="1" spans="1:9">
+      <c r="A27" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="B27" s="23" t="s">
+      <c r="B27" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="C27" s="23" t="s">
+      <c r="C27" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D27" s="24" t="s">
+      <c r="D27" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="E27" s="23" t="s">
+      <c r="E27" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="F27" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="G27" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="H27" s="23" t="s">
+      <c r="F27" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="G27" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="H27" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="I27" s="24" t="s">
+      <c r="I27" s="12" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="28" s="13" customFormat="1" spans="1:9">
-      <c r="A28" s="25" t="s">
+    <row r="28" s="14" customFormat="1" spans="1:9">
+      <c r="A28" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="B28" s="26" t="s">
+      <c r="B28" s="27" t="s">
         <v>103</v>
       </c>
-      <c r="C28" s="26" t="s">
+      <c r="C28" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="D28" s="27" t="s">
+      <c r="D28" s="28" t="s">
         <v>125</v>
       </c>
-      <c r="E28" s="26" t="s">
+      <c r="E28" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="F28" s="26" t="s">
+      <c r="F28" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="G28" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="H28" s="26" t="s">
+      <c r="G28" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="H28" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="I28" s="27" t="s">
+      <c r="I28" s="28" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="29" s="12" customFormat="1" spans="1:9">
-      <c r="A29" s="22" t="s">
+    <row r="29" s="13" customFormat="1" spans="1:9">
+      <c r="A29" s="24" t="s">
         <v>127</v>
       </c>
-      <c r="B29" s="23" t="s">
+      <c r="B29" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="C29" s="23" t="s">
+      <c r="C29" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D29" s="24" t="s">
+      <c r="D29" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="E29" s="23" t="s">
+      <c r="E29" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="F29" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="G29" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="H29" s="23" t="s">
+      <c r="F29" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="G29" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="H29" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="I29" s="24" t="s">
+      <c r="I29" s="12" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="30" s="14" customFormat="1" spans="1:9">
-      <c r="A30" s="28" t="s">
+    <row r="30" s="15" customFormat="1" spans="1:9">
+      <c r="A30" s="29" t="s">
         <v>130</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C30" s="29" t="s">
+      <c r="C30" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="D30" s="30" t="s">
+      <c r="D30" s="31" t="s">
         <v>131</v>
       </c>
-      <c r="E30" s="29" t="s">
+      <c r="E30" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="F30" s="29" t="s">
+      <c r="F30" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G30" s="29" t="s">
-        <v>6</v>
-      </c>
-      <c r="H30" s="29" t="s">
+      <c r="G30" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="H30" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="I30" s="30" t="s">
+      <c r="I30" s="31" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="31" s="15" customFormat="1" spans="1:9">
-      <c r="A31" s="31" t="s">
+    <row r="31" s="16" customFormat="1" spans="1:9">
+      <c r="A31" s="32" t="s">
         <v>133</v>
       </c>
-      <c r="B31" s="32" t="s">
+      <c r="B31" s="33" t="s">
         <v>103</v>
       </c>
-      <c r="C31" s="32" t="s">
+      <c r="C31" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="D31" s="33" t="s">
+      <c r="D31" s="34" t="s">
         <v>134</v>
       </c>
-      <c r="E31" s="32" t="s">
+      <c r="E31" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="F31" s="32" t="s">
+      <c r="F31" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="G31" s="32" t="s">
-        <v>6</v>
-      </c>
-      <c r="H31" s="32" t="s">
+      <c r="G31" s="33" t="s">
+        <v>6</v>
+      </c>
+      <c r="H31" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="I31" s="33" t="s">
+      <c r="I31" s="34" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="32" ht="25" spans="1:9">
-      <c r="A32" s="3" t="s">
+    <row r="32" s="17" customFormat="1" ht="25" spans="1:9">
+      <c r="A32" s="35" t="s">
         <v>136</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="36" t="s">
         <v>103</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="36" t="s">
         <v>54</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="D32" s="37" t="s">
         <v>137</v>
       </c>
-      <c r="E32" s="20" t="s">
+      <c r="E32" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="F32" s="5" t="s">
+      <c r="F32" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="G32" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H32" s="5" t="s">
+      <c r="G32" s="36" t="s">
+        <v>6</v>
+      </c>
+      <c r="H32" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="I32" s="4" t="s">
+      <c r="I32" s="37" t="s">
         <v>138</v>
       </c>
     </row>
@@ -3852,7 +3868,7 @@
       <c r="G34" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H34" s="16" t="s">
+      <c r="H34" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I34" s="4" t="s">
@@ -3881,7 +3897,7 @@
       <c r="G35" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H35" s="16" t="s">
+      <c r="H35" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I35" s="4" t="s">
@@ -3939,7 +3955,7 @@
       <c r="G37" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H37" s="16" t="s">
+      <c r="H37" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I37" s="4" t="s">
@@ -3983,7 +3999,7 @@
         <v>153</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>161</v>
@@ -3997,7 +4013,7 @@
       <c r="G39" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H39" s="16" t="s">
+      <c r="H39" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I39" s="4" t="s">
@@ -4862,7 +4878,7 @@
         <v>288</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>8</v>

</xml_diff>